<commit_message>
add encoder-only and clustering recommendation ablation experiments
</commit_message>
<xml_diff>
--- a/abalation/extended_ablation_table_with_novelty.xlsx
+++ b/abalation/extended_ablation_table_with_novelty.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M7"/>
+  <dimension ref="A1:M11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -693,80 +693,80 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>w/o EMA</t>
+          <t>PCL encoder only</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>573</v>
+        <v>404</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>0.1413 ± 0.0366</t>
+          <t>0.7286 ± 0.0457</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>7/7</t>
+          <t>3/7</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>0.6693</t>
+          <t>0.4044</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>0.3278 ± 0.1029</t>
+          <t>0.3794 ± 0.1127</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>0.6722 ± 0.1029</t>
+          <t>0.6206 ± 0.1127</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>1.22%</t>
+          <t>1.73%</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>12.91%</t>
+          <t>29.21%</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>85.86%</t>
+          <t>69.06%</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>0.8101</t>
+          <t>0.7755</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>1.8604%</t>
+          <t>1.3117%</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>0.2533</t>
+          <t>0.9689</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>w/o decorrelation</t>
+          <t>USL encoder only</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1741</v>
+        <v>1622</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>0.0807 ± 0.0149</t>
+          <t>0.0854 ± 0.0108</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -776,110 +776,370 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>0.0371</t>
+          <t>0.3495</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>0.3730 ± 0.0817</t>
+          <t>0.3677 ± 0.0889</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>0.6270 ± 0.0817</t>
+          <t>0.6323 ± 0.0889</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>0.75%</t>
+          <t>0.43%</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>30.21%</t>
+          <t>30.70%</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>69.04%</t>
+          <t>68.87%</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>0.7338</t>
+          <t>0.7517</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>5.6526%</t>
+          <t>5.2662%</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>-0.2245</t>
+          <t>-0.1852</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>PCL encoder clustering</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>341</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>0.5711 ± 0.1105</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>6/7</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>0.4266</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>0.3449 ± 0.0744</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>0.6551 ± 0.0744</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>22.29%</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>77.71%</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>0.7713</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>1.1071%</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>0.9160</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>USL encoder clustering</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>155</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>0.0799 ± 0.0212</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>4/7</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>0.2604</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>0.3238 ± 0.0607</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>0.6762 ± 0.0607</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>10.32%</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>89.68%</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>0.7673</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>0.5032%</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>0.7860</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>w/o EMA</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>573</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>0.1413 ± 0.0366</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>7/7</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>0.6693</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>0.3278 ± 0.1029</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>0.6722 ± 0.1029</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>1.22%</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>12.91%</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>85.86%</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>0.8101</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>1.8604%</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>0.2533</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>w/o decorrelation</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>1741</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>0.0807 ± 0.0149</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>4/7</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>0.0371</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>0.3730 ± 0.0817</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>0.6270 ± 0.0817</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>0.75%</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>30.21%</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>69.04%</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>0.7338</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>5.6526%</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>-0.2245</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
           <t>w/o top-K</t>
         </is>
       </c>
-      <c r="B7" t="n">
+      <c r="B11" t="n">
         <v>297</v>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>0.2572 ± 0.0000</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D11" t="inlineStr">
         <is>
           <t>1/7</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="E11" t="inlineStr">
         <is>
           <t>-0.0000</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="F11" t="inlineStr">
         <is>
           <t>0.3442 ± 0.2060</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="G11" t="inlineStr">
         <is>
           <t>0.6558 ± 0.2060</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="H11" t="inlineStr">
         <is>
           <t>7.07%</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="I11" t="inlineStr">
         <is>
           <t>23.91%</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="J11" t="inlineStr">
         <is>
           <t>69.02%</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr">
+      <c r="K11" t="inlineStr">
         <is>
           <t>0.8660</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr">
+      <c r="L11" t="inlineStr">
         <is>
           <t>0.9643%</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr">
+      <c r="M11" t="inlineStr">
         <is>
           <t>nan</t>
         </is>

</xml_diff>